<commit_message>
v 0.0.7 work in progress
</commit_message>
<xml_diff>
--- a/software/data_base/BD.xlsx
+++ b/software/data_base/BD.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29825"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{31511B1E-D1B9-4580-8A58-CE51DF4C67C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{64C628BE-CDA0-490D-BCDA-F4CE5D2B5D5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Params" sheetId="1" r:id="rId1"/>
@@ -2826,7 +2826,7 @@
         <v>0</v>
       </c>
       <c r="M43">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:13">
@@ -2908,7 +2908,7 @@
         <v>0</v>
       </c>
       <c r="M45">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:13">
@@ -2990,7 +2990,7 @@
         <v>0</v>
       </c>
       <c r="M47">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="48" spans="1:13">

</xml_diff>